<commit_message>
Add 55 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 653
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,28 +37,64 @@
     <t>url</t>
   </si>
   <si>
+    <t>en-in.report.json</t>
+  </si>
+  <si>
+    <t>["hero-video","columns-feature","columns-feature","cards-casestudy","cards-solutions","carousel-culture","cards-insights"]</t>
+  </si>
+  <si>
+    <t>en-in</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>homepage</t>
+  </si>
+  <si>
+    <t>2026-05-25T15:46:45.466Z</t>
+  </si>
+  <si>
+    <t>DEPT® | Growth Invention | Tech &amp; Marketing</t>
+  </si>
+  <si>
+    <t>https://www.deptagency.com/en-in/</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-homepage","columns","columns","cards-icon-links","hero-feature","cards"]</t>
+    <t>["hero-wizard","cards-callout","hero-promo","hero-promo","cards-article","cards-article","cards-product","hero-media","cards-video","carousel-badges"]</t>
   </si>
   <si>
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>homepage</t>
-  </si>
-  <si>
-    <t>2026-03-23T14:48:01.681Z</t>
-  </si>
-  <si>
-    <t>NGS Super: High-performing Industry Super Fund For Education</t>
-  </si>
-  <si>
-    <t>https://www.ngssuper.com.au/</t>
+    <t>2026-07-08T07:20:18.510Z</t>
+  </si>
+  <si>
+    <t>Wall Paint Colours - Home Painting, House Colour &amp; Paint Solutions | Dulux India</t>
+  </si>
+  <si>
+    <t>https://www.dulux.in/</t>
+  </si>
+  <si>
+    <t>project-gallery-photos.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>project-gallery-photos</t>
+  </si>
+  <si>
+    <t>gallery</t>
+  </si>
+  <si>
+    <t>2026-05-05T08:10:20.687Z</t>
+  </si>
+  <si>
+    <t>https://www.nprpl.com/project-gallery-photos</t>
   </si>
 </sst>
 </file>
@@ -447,16 +483,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="8" max="8" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +545,58 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>